<commit_message>
Archive unnecessary documentation and analysis scripts; restore create_hyperparameter_summary.R for methodology consolidation
</commit_message>
<xml_diff>
--- a/results/consolidated/Distributional_Metrics.xlsx
+++ b/results/consolidated/Distributional_Metrics.xlsx
@@ -444,10 +444,10 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0801949490474081</v>
+        <v>0.0821149017870329</v>
       </c>
       <c r="D2" t="n">
-        <v>0.157636568166926</v>
+        <v>0.156206358339881</v>
       </c>
       <c r="E2" t="n">
         <v>3.16745387149051</v>
@@ -470,7 +470,7 @@
         <v>0.065869147836361</v>
       </c>
       <c r="D3" t="n">
-        <v>0.136087191731774</v>
+        <v>0.136462363003612</v>
       </c>
       <c r="E3" t="n">
         <v>3.1500756077916</v>
@@ -490,10 +490,10 @@
         <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0550878747600059</v>
+        <v>0.0503618372470831</v>
       </c>
       <c r="D4" t="n">
-        <v>0.119678882643744</v>
+        <v>0.109570277748539</v>
       </c>
       <c r="E4" t="n">
         <v>3.24083533075908</v>
@@ -513,10 +513,10 @@
         <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0769457982572737</v>
+        <v>0.0803426377196869</v>
       </c>
       <c r="D5" t="n">
-        <v>0.174195601774061</v>
+        <v>0.174467468214253</v>
       </c>
       <c r="E5" t="n">
         <v>2.73031669669996</v>
@@ -536,19 +536,19 @@
         <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0686752326096588</v>
+        <v>0.0663122138531975</v>
       </c>
       <c r="D6" t="n">
-        <v>0.164512008143137</v>
+        <v>0.159749891039588</v>
       </c>
       <c r="E6" t="n">
-        <v>2.95319480751647</v>
+        <v>2.95319480751651</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.290767344618739</v>
+        <v>-0.290767344618738</v>
       </c>
       <c r="G6" t="n">
-        <v>17.5934929069273</v>
+        <v>17.5934929069274</v>
       </c>
     </row>
     <row r="7">
@@ -559,10 +559,10 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0824102791315906</v>
+        <v>0.0939299955693398</v>
       </c>
       <c r="D7" t="n">
-        <v>0.209776640279721</v>
+        <v>0.219618266406986</v>
       </c>
       <c r="E7" t="n">
         <v>2.60571749545656</v>
@@ -582,10 +582,10 @@
         <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>0.304829419583518</v>
+        <v>0.310146211785556</v>
       </c>
       <c r="D8" t="n">
-        <v>0.608208859026904</v>
+        <v>0.602427639066635</v>
       </c>
       <c r="E8" t="n">
         <v>1.23795205887821</v>
@@ -605,10 +605,10 @@
         <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>0.344040762073549</v>
+        <v>0.334514842711564</v>
       </c>
       <c r="D9" t="n">
-        <v>0.668035615819896</v>
+        <v>0.666307752543019</v>
       </c>
       <c r="E9" t="n">
         <v>1.07904672660092</v>
@@ -627,21 +627,11 @@
       <c r="B10" t="s">
         <v>10</v>
       </c>
-      <c r="C10" t="n">
-        <v>0.0298331118003249</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.0581859466874666</v>
-      </c>
-      <c r="E10" t="n">
-        <v>3.72044075198291</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.470402467111507</v>
-      </c>
-      <c r="G10" t="n">
-        <v>4.17017071750532</v>
-      </c>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+      <c r="G10"/>
     </row>
     <row r="11">
       <c r="A11" t="s">
@@ -651,19 +641,19 @@
         <v>11</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0540540540540541</v>
+        <v>0.163491360212672</v>
       </c>
       <c r="D11" t="n">
-        <v>0.14113158447845</v>
+        <v>0.236785111906135</v>
       </c>
       <c r="E11" t="n">
-        <v>2.89990750691682</v>
+        <v>3.91037315514876</v>
       </c>
       <c r="F11" t="n">
-        <v>0.548908556313725</v>
+        <v>-1.87959438539939</v>
       </c>
       <c r="G11" t="n">
-        <v>17.3002692609863</v>
+        <v>13.1827363509551</v>
       </c>
     </row>
     <row r="12">
@@ -673,21 +663,11 @@
       <c r="B12" t="s">
         <v>12</v>
       </c>
-      <c r="C12" t="n">
-        <v>0.0642445724412938</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0.149860776530063</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2.88268362373451</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0.118318091282215</v>
-      </c>
-      <c r="G12" t="n">
-        <v>12.9374659452236</v>
-      </c>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
     </row>
     <row r="13">
       <c r="A13" t="s">
@@ -696,21 +676,11 @@
       <c r="B13" t="s">
         <v>13</v>
       </c>
-      <c r="C13" t="n">
-        <v>0.0599616009452075</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.167481256957086</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2.60404643848225</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1.17076818961658</v>
-      </c>
-      <c r="G13" t="n">
-        <v>21.606779230327</v>
-      </c>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
     </row>
     <row r="14">
       <c r="A14" t="s">
@@ -720,10 +690,10 @@
         <v>8</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0998375424604933</v>
+        <v>0.0958499483089647</v>
       </c>
       <c r="D14" t="n">
-        <v>0.210827810171211</v>
+        <v>0.208802205050974</v>
       </c>
       <c r="E14" t="n">
         <v>2.80686466616841</v>
@@ -743,10 +713,10 @@
         <v>9</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0954068822921282</v>
+        <v>0.0899424014178112</v>
       </c>
       <c r="D15" t="n">
-        <v>0.208098918338524</v>
+        <v>0.207561420642828</v>
       </c>
       <c r="E15" t="n">
         <v>2.45210132213632</v>
@@ -766,10 +736,10 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0700044306601684</v>
+        <v>0.0704474966770049</v>
       </c>
       <c r="D16" t="n">
-        <v>0.167467331084733</v>
+        <v>0.163173855721279</v>
       </c>
       <c r="E16" t="n">
         <v>2.80984099881588</v>
@@ -789,19 +759,19 @@
         <v>11</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0998375424604933</v>
+        <v>0.102052872544676</v>
       </c>
       <c r="D17" t="n">
-        <v>0.225404071214227</v>
+        <v>0.225304617973403</v>
       </c>
       <c r="E17" t="n">
         <v>2.50881375230642</v>
       </c>
       <c r="F17" t="n">
-        <v>1.74401935510357</v>
+        <v>1.74401935510359</v>
       </c>
       <c r="G17" t="n">
-        <v>33.9540592100708</v>
+        <v>33.9540592100711</v>
       </c>
     </row>
     <row r="18">
@@ -812,10 +782,10 @@
         <v>12</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0954068822921282</v>
+        <v>0.0911239107960419</v>
       </c>
       <c r="D18" t="n">
-        <v>0.216318983199867</v>
+        <v>0.215774827694079</v>
       </c>
       <c r="E18" t="n">
         <v>2.64500822858612</v>
@@ -835,10 +805,10 @@
         <v>13</v>
       </c>
       <c r="C19" t="n">
-        <v>0.111948013587358</v>
+        <v>0.111800324915079</v>
       </c>
       <c r="D19" t="n">
-        <v>0.266266426416811</v>
+        <v>0.260317717474662</v>
       </c>
       <c r="E19" t="n">
         <v>2.31734724008197</v>
@@ -858,10 +828,10 @@
         <v>8</v>
       </c>
       <c r="C20" t="n">
-        <v>0.0497710825579678</v>
+        <v>0.0451927337173239</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0936113993413482</v>
+        <v>0.0938271338711843</v>
       </c>
       <c r="E20" t="n">
         <v>3.30362050153608</v>
@@ -881,10 +851,10 @@
         <v>9</v>
       </c>
       <c r="C21" t="n">
-        <v>0.0364791020528725</v>
+        <v>0.0443066016836509</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0792599135831264</v>
+        <v>0.0860304627306064</v>
       </c>
       <c r="E21" t="n">
         <v>3.55462703307353</v>
@@ -904,10 +874,10 @@
         <v>10</v>
       </c>
       <c r="C22" t="n">
-        <v>0.176044897356373</v>
+        <v>0.173091123910796</v>
       </c>
       <c r="D22" t="n">
-        <v>0.24600444516633</v>
+        <v>0.248869546555533</v>
       </c>
       <c r="E22" t="n">
         <v>3.38654768167346</v>
@@ -927,19 +897,19 @@
         <v>11</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0527248560035445</v>
+        <v>0.0573032048441885</v>
       </c>
       <c r="D23" t="n">
-        <v>0.14141188223432</v>
+        <v>0.144488812362079</v>
       </c>
       <c r="E23" t="n">
-        <v>2.84506444426865</v>
+        <v>2.84506444423159</v>
       </c>
       <c r="F23" t="n">
-        <v>0.736277432094375</v>
+        <v>0.736277432110608</v>
       </c>
       <c r="G23" t="n">
-        <v>17.7952620064131</v>
+        <v>17.7952620065376</v>
       </c>
     </row>
     <row r="24">
@@ -950,19 +920,19 @@
         <v>12</v>
       </c>
       <c r="C24" t="n">
-        <v>0.0573032048441885</v>
+        <v>0.0575985821887461</v>
       </c>
       <c r="D24" t="n">
-        <v>0.141145606787678</v>
+        <v>0.13815579128666</v>
       </c>
       <c r="E24" t="n">
-        <v>2.96328437147108</v>
+        <v>2.96328437151777</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.334887482435224</v>
+        <v>-0.334887482419656</v>
       </c>
       <c r="G24" t="n">
-        <v>13.4862683618879</v>
+        <v>13.4862683618155</v>
       </c>
     </row>
     <row r="25">
@@ -973,10 +943,10 @@
         <v>13</v>
       </c>
       <c r="C25" t="n">
-        <v>0.0691182986264954</v>
+        <v>0.0666075911977551</v>
       </c>
       <c r="D25" t="n">
-        <v>0.179050301542886</v>
+        <v>0.180971508720854</v>
       </c>
       <c r="E25" t="n">
         <v>2.58537455920498</v>
@@ -1030,22 +1000,22 @@
         <v>15</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0954068822921282</v>
+        <v>0.0935361591099296</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0976222123763107</v>
+        <v>0.0934869295525033</v>
       </c>
       <c r="D2" t="n">
-        <v>0.215730590070896</v>
+        <v>0.213489107426204</v>
       </c>
       <c r="E2" t="n">
-        <v>0.213573396685539</v>
+        <v>0.212288516372527</v>
       </c>
       <c r="F2" t="n">
         <v>2.58999603468252</v>
       </c>
       <c r="G2" t="n">
-        <v>0.424905513461851</v>
+        <v>0.424905513461854</v>
       </c>
       <c r="H2" t="n">
         <v>27.86455188624</v>
@@ -1056,25 +1026,25 @@
         <v>14</v>
       </c>
       <c r="B3" t="n">
-        <v>0.142827253482991</v>
+        <v>0.269384138236597</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0621030866932506</v>
+        <v>0.310146211785556</v>
       </c>
       <c r="D3" t="n">
-        <v>0.298817339916644</v>
+        <v>0.501840167838596</v>
       </c>
       <c r="E3" t="n">
-        <v>0.158671016743574</v>
+        <v>0.602427639066635</v>
       </c>
       <c r="F3" t="n">
-        <v>2.40401285109927</v>
+        <v>2.07579064687596</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.0111743714512416</v>
+        <v>-1.41834597281029</v>
       </c>
       <c r="H3" t="n">
-        <v>79.0060012353707</v>
+        <v>143.734686203046</v>
       </c>
     </row>
     <row r="4">
@@ -1082,25 +1052,25 @@
         <v>16</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0735735735735736</v>
+        <v>0.0740166395904101</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0550140304238665</v>
+        <v>0.0574508935164673</v>
       </c>
       <c r="D4" t="n">
-        <v>0.146747258109281</v>
+        <v>0.148723875921153</v>
       </c>
       <c r="E4" t="n">
-        <v>0.141278744510999</v>
+        <v>0.14132230182437</v>
       </c>
       <c r="F4" t="n">
-        <v>3.10641976520463</v>
+        <v>3.10641976520623</v>
       </c>
       <c r="G4" t="n">
-        <v>0.199479356316453</v>
+        <v>0.199479356321753</v>
       </c>
       <c r="H4" t="n">
-        <v>13.0226291819186</v>
+        <v>13.0226291819273</v>
       </c>
     </row>
     <row r="5">
@@ -1108,16 +1078,16 @@
         <v>7</v>
       </c>
       <c r="B5" t="n">
-        <v>0.071530546940383</v>
+        <v>0.0731551223354502</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0728105154334663</v>
+        <v>0.0733274257864422</v>
       </c>
       <c r="D5" t="n">
-        <v>0.160314482123227</v>
+        <v>0.159345770792143</v>
       </c>
       <c r="E5" t="n">
-        <v>0.161074288155032</v>
+        <v>0.157978124689735</v>
       </c>
       <c r="F5" t="n">
         <v>2.9745989682857</v>

</xml_diff>